<commit_message>
Correct independent coding provenance
</commit_message>
<xml_diff>
--- a/research/structural-profiles-pilot/submissions/independent/independent_submission_v1.xlsx
+++ b/research/structural-profiles-pilot/submissions/independent/independent_submission_v1.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1_S5_RUBRIC" sheetId="1" r:id="Rced87a6542774305"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCOPE_REFERENCE" sheetId="2" r:id="R12b765aeebd14a53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUBMISSION" sheetId="3" r:id="Re84474b670624e7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S1_S5_RUBRIC" sheetId="1" r:id="R8285a0d2eebc43a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCOPE_REFERENCE" sheetId="2" r:id="R183a1feae39d43f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUBMISSION" sheetId="3" r:id="R834df17ab6a44349"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -952,7 +952,7 @@
     <x:mergeCell ref="A1:G1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78136c2ae8bd44dd"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88f7d56138ff4fa5"/>
 </x:worksheet>
 </file>
 
@@ -2327,7 +2327,7 @@
     <x:mergeCell ref="A1:H1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4f02ac1076954e9a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4d262ef3ab64385"/>
 </x:worksheet>
 </file>
 
@@ -2564,7 +2564,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N4" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O4" s="4" t="n">
         <x:v>4</x:v>
@@ -2598,7 +2598,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z4" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports mature-software requirements and architecture.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports mature-software requirements and architecture.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="36" customHeight="1">
@@ -2662,7 +2662,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N5" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O5" s="4" t="n">
         <x:v>4</x:v>
@@ -2696,7 +2696,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z5" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports mature-software implementation.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports mature-software implementation.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="36" customHeight="1">
@@ -2760,7 +2760,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N6" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O6" s="4" t="n">
         <x:v>4</x:v>
@@ -2794,7 +2794,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z6" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports mature-software verification and validation.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports mature-software verification and validation.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="36" customHeight="1">
@@ -2858,7 +2858,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N7" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O7" s="4" t="n">
         <x:v>3</x:v>
@@ -2892,7 +2892,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z7" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports mature-software deployment.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports mature-software deployment.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="36" customHeight="1">
@@ -2956,7 +2956,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N8" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O8" s="4" t="n">
         <x:v>4</x:v>
@@ -2990,7 +2990,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z8" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports mature-software operations and maintenance.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports mature-software operations and maintenance.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="36" customHeight="1">
@@ -3054,7 +3054,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N9" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O9" s="4" t="n">
         <x:v>3</x:v>
@@ -3088,7 +3088,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z9" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports discrete-manufacturing product design.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports discrete-manufacturing product design.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="36" customHeight="1">
@@ -3152,7 +3152,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N10" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O10" s="4" t="n">
         <x:v>2</x:v>
@@ -3186,7 +3186,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z10" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports discrete-manufacturing process engineering.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports discrete-manufacturing process engineering.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
@@ -3250,7 +3250,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N11" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O11" s="4" t="n">
         <x:v>1</x:v>
@@ -3284,7 +3284,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z11" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports scoped supply and tooling readiness.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports scoped supply and tooling readiness.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="36" customHeight="1">
@@ -3348,7 +3348,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N12" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O12" s="4" t="n">
         <x:v>1</x:v>
@@ -3382,7 +3382,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z12" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports discrete-manufacturing retooling and commissioning.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports discrete-manufacturing retooling and commissioning.</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="36" customHeight="1">
@@ -3446,7 +3446,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N13" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O13" s="4" t="n">
         <x:v>4</x:v>
@@ -3480,7 +3480,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z13" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports discrete-manufacturing production planning and scheduling.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports discrete-manufacturing production planning and scheduling.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="36" customHeight="1">
@@ -3544,7 +3544,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N14" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O14" s="4" t="n">
         <x:v>2</x:v>
@@ -3578,7 +3578,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z14" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports scoped production and process control.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports scoped production and process control.</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="36" customHeight="1">
@@ -3642,7 +3642,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N15" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O15" s="4" t="n">
         <x:v>2</x:v>
@@ -3676,7 +3676,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z15" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports scoped discrete-manufacturing quality assurance.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports scoped discrete-manufacturing quality assurance.</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="36" customHeight="1">
@@ -3740,7 +3740,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N16" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O16" s="4" t="n">
         <x:v>2</x:v>
@@ -3774,7 +3774,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z16" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports maintenance and continuous improvement in the frozen pathway.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports maintenance and continuous improvement in the frozen pathway.</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="36" customHeight="1">
@@ -3838,7 +3838,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N17" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O17" s="4" t="n">
         <x:v>4</x:v>
@@ -3872,7 +3872,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z17" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports pilot-relevant tokamak theory and system design.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports pilot-relevant tokamak theory and system design.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="36" customHeight="1">
@@ -3936,7 +3936,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N18" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O18" s="4" t="n">
         <x:v>4</x:v>
@@ -3970,7 +3970,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z18" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports scoped tokamak simulation.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports scoped tokamak simulation.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="36" customHeight="1">
@@ -4034,7 +4034,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N19" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O19" s="4" t="n">
         <x:v>4</x:v>
@@ -4068,7 +4068,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z19" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports tokamak experiment selection and shot-throughput constraints.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports tokamak experiment selection and shot-throughput constraints.</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="36" customHeight="1">
@@ -4132,7 +4132,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N20" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O20" s="4" t="n">
         <x:v>2</x:v>
@@ -4166,7 +4166,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z20" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports pilot-relevant tokamak diagnostics.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports pilot-relevant tokamak diagnostics.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="36" customHeight="1">
@@ -4230,7 +4230,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N21" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O21" s="4" t="n">
         <x:v>2</x:v>
@@ -4264,7 +4264,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z21" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports tokamak plasma-control development and live testing.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports tokamak plasma-control development and live testing.</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="36" customHeight="1">
@@ -4328,7 +4328,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N22" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O22" s="4" t="n">
         <x:v>2</x:v>
@@ -4362,7 +4362,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z22" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports tokamak materials discovery and screening.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports tokamak materials discovery and screening.</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="36" customHeight="1">
@@ -4426,7 +4426,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N23" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O23" s="4" t="n">
         <x:v>0</x:v>
@@ -4460,7 +4460,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z23" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports pilot-relevant tokamak materials qualification.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports pilot-relevant tokamak materials qualification.</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="36" customHeight="1">
@@ -4524,7 +4524,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N24" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O24" s="4" t="n">
         <x:v>2</x:v>
@@ -4558,7 +4558,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z24" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports pilot-relevant tokamak magnet development.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports pilot-relevant tokamak magnet development.</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="36" customHeight="1">
@@ -4622,7 +4622,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N25" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O25" s="4" t="n">
         <x:v>2</x:v>
@@ -4656,7 +4656,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z25" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports pilot-relevant heating and current-drive development.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports pilot-relevant heating and current-drive development.</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="36" customHeight="1">
@@ -4720,7 +4720,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N26" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O26" s="4" t="n">
         <x:v>2</x:v>
@@ -4754,7 +4754,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z26" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports pilot-relevant plasma-facing component development.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports pilot-relevant plasma-facing component development.</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="36" customHeight="1">
@@ -4818,7 +4818,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N27" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O27" s="4" t="n">
         <x:v>1</x:v>
@@ -4852,7 +4852,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z27" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports pilot-relevant tritium and fuel-cycle development.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports pilot-relevant tritium and fuel-cycle development.</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="36" customHeight="1">
@@ -4916,7 +4916,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N28" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O28" s="4" t="n">
         <x:v>2</x:v>
@@ -4950,7 +4950,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z28" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports pilot-relevant tokamak blanket development.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports pilot-relevant tokamak blanket development.</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="36" customHeight="1">
@@ -5014,7 +5014,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N29" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O29" s="4" t="n">
         <x:v>0</x:v>
@@ -5048,7 +5048,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z29" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports pilot-relevant tokamak component fabrication.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports pilot-relevant tokamak component fabrication.</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="36" customHeight="1">
@@ -5112,7 +5112,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N30" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O30" s="4" t="n">
         <x:v>0</x:v>
@@ -5146,7 +5146,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z30" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports pilot-relevant tokamak facility construction.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports pilot-relevant tokamak facility construction.</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="36" customHeight="1">
@@ -5210,7 +5210,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N31" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O31" s="4" t="n">
         <x:v>1</x:v>
@@ -5244,7 +5244,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z31" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports pilot-relevant tokamak commissioning.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports pilot-relevant tokamak commissioning.</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="36" customHeight="1">
@@ -5308,7 +5308,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N32" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O32" s="4" t="n">
         <x:v>0</x:v>
@@ -5342,7 +5342,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z32" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports pilot-relevant tokamak reliability demonstration.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports pilot-relevant tokamak reliability demonstration.</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="36" customHeight="1">
@@ -5406,7 +5406,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N33" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O33" s="4" t="n">
         <x:v>4</x:v>
@@ -5440,7 +5440,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z33" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports pilot-relevant tokamak licensing.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports pilot-relevant tokamak licensing.</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="36" customHeight="1">
@@ -5504,7 +5504,7 @@
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="N34" s="4" t="str">
-        <x:v>model_identifier_not_exposed</x:v>
+        <x:v>gpt-5.6</x:v>
       </x:c>
       <x:c r="O34" s="4" t="n">
         <x:v>2</x:v>
@@ -5538,7 +5538,7 @@
         <x:v>submitted</x:v>
       </x:c>
       <x:c r="Z34" s="4" t="str">
-        <x:v>runtime limitation: exact model identifier not exposed; source_gap: no canonical source directly supports tokamak pilot grid integration.</x:v>
+        <x:v>reasoning_effort=extra_high; model provenance supplied by owner after task completion; source_gap: no canonical source directly supports tokamak pilot grid integration.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5581,6 +5581,6 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0b5a0ceb15024cd0"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7ce9cca37de44af"/>
 </x:worksheet>
 </file>
</xml_diff>